<commit_message>
Separar jornadas por rangos de fechas semanales en hojas individuales de Excel
</commit_message>
<xml_diff>
--- a/data/Premier.xlsx
+++ b/data/Premier.xlsx
@@ -32,13 +32,23 @@
     <sheet sheetId="12" name="Jornada 36" state="visible" r:id="rId26"/>
     <sheet sheetId="13" name="Jornada 37" state="visible" r:id="rId27"/>
     <sheet sheetId="14" name="Jornada 38" state="visible" r:id="rId28"/>
+    <sheet sheetId="26" name="21.08.2026 - 24.08.2026" state="visible" r:id="rId29"/>
+    <sheet sheetId="27" name="28.08.2026 - 31.08.2026" state="visible" r:id="rId30"/>
+    <sheet sheetId="28" name="04.09.2026 - 06.09.2026" state="visible" r:id="rId31"/>
+    <sheet sheetId="29" name="12.09.2026 - 14.09.2026" state="visible" r:id="rId32"/>
+    <sheet sheetId="30" name="18.09.2026 - 20.09.2026" state="visible" r:id="rId33"/>
+    <sheet sheetId="31" name="10.10.2026 - 12.10.2026" state="visible" r:id="rId34"/>
+    <sheet sheetId="32" name="17.10.2026 - 19.10.2026" state="visible" r:id="rId35"/>
+    <sheet sheetId="33" name="23.10.2026 - 25.10.2026" state="visible" r:id="rId36"/>
+    <sheet sheetId="34" name="31.10.2026 - 02.11.2026" state="visible" r:id="rId37"/>
+    <sheet sheetId="35" name="07.11.2026" state="visible" r:id="rId38"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1736" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2506" uniqueCount="211">
   <si>
     <t>Matchday</t>
   </si>
@@ -542,6 +552,135 @@
   </si>
   <si>
     <t>28/12/2025</t>
+  </si>
+  <si>
+    <t>Fechas 21/08/2026 - 24/08/2026</t>
+  </si>
+  <si>
+    <t>21/08/2026</t>
+  </si>
+  <si>
+    <t>Coventry City</t>
+  </si>
+  <si>
+    <t>22/08/2026</t>
+  </si>
+  <si>
+    <t>Hull City</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>23/08/2026</t>
+  </si>
+  <si>
+    <t>24/08/2026</t>
+  </si>
+  <si>
+    <t>Fechas 28/08/2026 - 31/08/2026</t>
+  </si>
+  <si>
+    <t>28/08/2026</t>
+  </si>
+  <si>
+    <t>29/08/2026</t>
+  </si>
+  <si>
+    <t>30/08/2026</t>
+  </si>
+  <si>
+    <t>31/08/2026</t>
+  </si>
+  <si>
+    <t>Fechas 04/09/2026 - 06/09/2026</t>
+  </si>
+  <si>
+    <t>04/09/2026</t>
+  </si>
+  <si>
+    <t>05/09/2026</t>
+  </si>
+  <si>
+    <t>06/09/2026</t>
+  </si>
+  <si>
+    <t>Fechas 12/09/2026 - 14/09/2026</t>
+  </si>
+  <si>
+    <t>12/09/2026</t>
+  </si>
+  <si>
+    <t>13/09/2026</t>
+  </si>
+  <si>
+    <t>14/09/2026</t>
+  </si>
+  <si>
+    <t>Fechas 18/09/2026 - 20/09/2026</t>
+  </si>
+  <si>
+    <t>18/09/2026</t>
+  </si>
+  <si>
+    <t>19/09/2026</t>
+  </si>
+  <si>
+    <t>20/09/2026</t>
+  </si>
+  <si>
+    <t>Fechas 10/10/2026 - 12/10/2026</t>
+  </si>
+  <si>
+    <t>10/10/2026</t>
+  </si>
+  <si>
+    <t>11/10/2026</t>
+  </si>
+  <si>
+    <t>12/10/2026</t>
+  </si>
+  <si>
+    <t>Fechas 17/10/2026 - 19/10/2026</t>
+  </si>
+  <si>
+    <t>17/10/2026</t>
+  </si>
+  <si>
+    <t>18/10/2026</t>
+  </si>
+  <si>
+    <t>19/10/2026</t>
+  </si>
+  <si>
+    <t>Fechas 23/10/2026 - 25/10/2026</t>
+  </si>
+  <si>
+    <t>23/10/2026</t>
+  </si>
+  <si>
+    <t>24/10/2026</t>
+  </si>
+  <si>
+    <t>25/10/2026</t>
+  </si>
+  <si>
+    <t>Fechas 31/10/2026 - 02/11/2026</t>
+  </si>
+  <si>
+    <t>31/10/2026</t>
+  </si>
+  <si>
+    <t>01/11/2026</t>
+  </si>
+  <si>
+    <t>02/11/2026</t>
+  </si>
+  <si>
+    <t>Fecha 07/11/2026</t>
+  </si>
+  <si>
+    <t>07/11/2026</t>
   </si>
 </sst>
 </file>
@@ -2553,7 +2692,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -5200,6 +5339,1094 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="32" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C2" t="s">
+        <v>169</v>
+      </c>
+      <c r="D2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>170</v>
+      </c>
+      <c r="G2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>168</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>171</v>
+      </c>
+      <c r="D3" t="s">
+        <v>106</v>
+      </c>
+      <c r="E3" t="s">
+        <v>172</v>
+      </c>
+      <c r="F3" t="s">
+        <v>45</v>
+      </c>
+      <c r="G3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>168</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>171</v>
+      </c>
+      <c r="D4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" t="s">
+        <v>28</v>
+      </c>
+      <c r="G4" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>168</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>171</v>
+      </c>
+      <c r="D5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" t="s">
+        <v>41</v>
+      </c>
+      <c r="F5" t="s">
+        <v>107</v>
+      </c>
+      <c r="G5" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>168</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>171</v>
+      </c>
+      <c r="D6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" t="s">
+        <v>50</v>
+      </c>
+      <c r="F6" t="s">
+        <v>108</v>
+      </c>
+      <c r="G6" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>168</v>
+      </c>
+      <c r="B7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" t="s">
+        <v>171</v>
+      </c>
+      <c r="D7" t="s">
+        <v>43</v>
+      </c>
+      <c r="E7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G7" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>168</v>
+      </c>
+      <c r="B8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" t="s">
+        <v>174</v>
+      </c>
+      <c r="D8" t="s">
+        <v>110</v>
+      </c>
+      <c r="E8" t="s">
+        <v>36</v>
+      </c>
+      <c r="F8" t="s">
+        <v>25</v>
+      </c>
+      <c r="G8" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>168</v>
+      </c>
+      <c r="B9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" t="s">
+        <v>174</v>
+      </c>
+      <c r="D9" t="s">
+        <v>110</v>
+      </c>
+      <c r="E9" t="s">
+        <v>31</v>
+      </c>
+      <c r="F9" t="s">
+        <v>22</v>
+      </c>
+      <c r="G9" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>168</v>
+      </c>
+      <c r="B10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" t="s">
+        <v>174</v>
+      </c>
+      <c r="D10" t="s">
+        <v>112</v>
+      </c>
+      <c r="E10" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" t="s">
+        <v>44</v>
+      </c>
+      <c r="G10" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>168</v>
+      </c>
+      <c r="B11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" t="s">
+        <v>175</v>
+      </c>
+      <c r="D11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F11" t="s">
+        <v>29</v>
+      </c>
+      <c r="G11" t="s">
+        <v>173</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="32" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>176</v>
+      </c>
+      <c r="B2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C2" t="s">
+        <v>177</v>
+      </c>
+      <c r="D2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F2" t="s">
+        <v>31</v>
+      </c>
+      <c r="G2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>176</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>178</v>
+      </c>
+      <c r="D3" t="s">
+        <v>106</v>
+      </c>
+      <c r="E3" t="s">
+        <v>44</v>
+      </c>
+      <c r="F3" t="s">
+        <v>50</v>
+      </c>
+      <c r="G3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>176</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>178</v>
+      </c>
+      <c r="D4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>176</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>178</v>
+      </c>
+      <c r="D5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" t="s">
+        <v>170</v>
+      </c>
+      <c r="F5" t="s">
+        <v>172</v>
+      </c>
+      <c r="G5" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>176</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>178</v>
+      </c>
+      <c r="D6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G6" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>176</v>
+      </c>
+      <c r="B7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" t="s">
+        <v>179</v>
+      </c>
+      <c r="D7" t="s">
+        <v>110</v>
+      </c>
+      <c r="E7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>176</v>
+      </c>
+      <c r="B8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" t="s">
+        <v>179</v>
+      </c>
+      <c r="D8" t="s">
+        <v>110</v>
+      </c>
+      <c r="E8" t="s">
+        <v>108</v>
+      </c>
+      <c r="F8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>176</v>
+      </c>
+      <c r="B9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" t="s">
+        <v>179</v>
+      </c>
+      <c r="D9" t="s">
+        <v>110</v>
+      </c>
+      <c r="E9" t="s">
+        <v>107</v>
+      </c>
+      <c r="F9" t="s">
+        <v>40</v>
+      </c>
+      <c r="G9" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>176</v>
+      </c>
+      <c r="B10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" t="s">
+        <v>179</v>
+      </c>
+      <c r="D10" t="s">
+        <v>112</v>
+      </c>
+      <c r="E10" t="s">
+        <v>45</v>
+      </c>
+      <c r="F10" t="s">
+        <v>41</v>
+      </c>
+      <c r="G10" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>176</v>
+      </c>
+      <c r="B11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" t="s">
+        <v>180</v>
+      </c>
+      <c r="D11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E11" t="s">
+        <v>25</v>
+      </c>
+      <c r="F11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" t="s">
+        <v>173</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="32" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>181</v>
+      </c>
+      <c r="B2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C2" t="s">
+        <v>182</v>
+      </c>
+      <c r="D2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F2" t="s">
+        <v>44</v>
+      </c>
+      <c r="G2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>181</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>183</v>
+      </c>
+      <c r="D3" t="s">
+        <v>106</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>181</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>183</v>
+      </c>
+      <c r="D4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" t="s">
+        <v>107</v>
+      </c>
+      <c r="G4" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>181</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>183</v>
+      </c>
+      <c r="D5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F5" t="s">
+        <v>108</v>
+      </c>
+      <c r="G5" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>181</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>183</v>
+      </c>
+      <c r="D6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F6" t="s">
+        <v>28</v>
+      </c>
+      <c r="G6" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>181</v>
+      </c>
+      <c r="B7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" t="s">
+        <v>183</v>
+      </c>
+      <c r="D7" t="s">
+        <v>39</v>
+      </c>
+      <c r="E7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" t="s">
+        <v>170</v>
+      </c>
+      <c r="G7" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>181</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" t="s">
+        <v>183</v>
+      </c>
+      <c r="D8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E8" t="s">
+        <v>50</v>
+      </c>
+      <c r="F8" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>181</v>
+      </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" t="s">
+        <v>183</v>
+      </c>
+      <c r="D9" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9" t="s">
+        <v>172</v>
+      </c>
+      <c r="F9" t="s">
+        <v>25</v>
+      </c>
+      <c r="G9" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>181</v>
+      </c>
+      <c r="B10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" t="s">
+        <v>184</v>
+      </c>
+      <c r="D10" t="s">
+        <v>110</v>
+      </c>
+      <c r="E10" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10" t="s">
+        <v>45</v>
+      </c>
+      <c r="G10" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>181</v>
+      </c>
+      <c r="B11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" t="s">
+        <v>184</v>
+      </c>
+      <c r="D11" t="s">
+        <v>112</v>
+      </c>
+      <c r="E11" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" t="s">
+        <v>29</v>
+      </c>
+      <c r="G11" t="s">
+        <v>173</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="32" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" t="s">
+        <v>186</v>
+      </c>
+      <c r="D2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>185</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>186</v>
+      </c>
+      <c r="D3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" t="s">
+        <v>50</v>
+      </c>
+      <c r="G3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>185</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>186</v>
+      </c>
+      <c r="D4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" t="s">
+        <v>172</v>
+      </c>
+      <c r="G4" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>185</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>186</v>
+      </c>
+      <c r="D5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G5" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>185</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>186</v>
+      </c>
+      <c r="D6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" t="s">
+        <v>44</v>
+      </c>
+      <c r="F6" t="s">
+        <v>40</v>
+      </c>
+      <c r="G6" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>185</v>
+      </c>
+      <c r="B7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" t="s">
+        <v>186</v>
+      </c>
+      <c r="D7" t="s">
+        <v>43</v>
+      </c>
+      <c r="E7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F7" t="s">
+        <v>23</v>
+      </c>
+      <c r="G7" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>185</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" t="s">
+        <v>186</v>
+      </c>
+      <c r="D8" t="s">
+        <v>66</v>
+      </c>
+      <c r="E8" t="s">
+        <v>107</v>
+      </c>
+      <c r="F8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>185</v>
+      </c>
+      <c r="B9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" t="s">
+        <v>187</v>
+      </c>
+      <c r="D9" t="s">
+        <v>110</v>
+      </c>
+      <c r="E9" t="s">
+        <v>170</v>
+      </c>
+      <c r="F9" t="s">
+        <v>36</v>
+      </c>
+      <c r="G9" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>185</v>
+      </c>
+      <c r="B10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" t="s">
+        <v>187</v>
+      </c>
+      <c r="D10" t="s">
+        <v>112</v>
+      </c>
+      <c r="E10" t="s">
+        <v>45</v>
+      </c>
+      <c r="F10" t="s">
+        <v>31</v>
+      </c>
+      <c r="G10" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>185</v>
+      </c>
+      <c r="B11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" t="s">
+        <v>188</v>
+      </c>
+      <c r="D11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E11" t="s">
+        <v>108</v>
+      </c>
+      <c r="F11" t="s">
+        <v>19</v>
+      </c>
+      <c r="G11" t="s">
+        <v>173</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G11"/>
@@ -5469,6 +6696,1638 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="32" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>189</v>
+      </c>
+      <c r="B2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C2" t="s">
+        <v>190</v>
+      </c>
+      <c r="D2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>189</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>191</v>
+      </c>
+      <c r="D3" t="s">
+        <v>106</v>
+      </c>
+      <c r="E3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>189</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>191</v>
+      </c>
+      <c r="D4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>189</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>191</v>
+      </c>
+      <c r="D5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G5" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>189</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>191</v>
+      </c>
+      <c r="D6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" t="s">
+        <v>108</v>
+      </c>
+      <c r="F6" t="s">
+        <v>28</v>
+      </c>
+      <c r="G6" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>189</v>
+      </c>
+      <c r="B7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" t="s">
+        <v>191</v>
+      </c>
+      <c r="D7" t="s">
+        <v>39</v>
+      </c>
+      <c r="E7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" t="s">
+        <v>107</v>
+      </c>
+      <c r="G7" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>189</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" t="s">
+        <v>191</v>
+      </c>
+      <c r="D8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" t="s">
+        <v>172</v>
+      </c>
+      <c r="G8" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>189</v>
+      </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" t="s">
+        <v>191</v>
+      </c>
+      <c r="D9" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9" t="s">
+        <v>50</v>
+      </c>
+      <c r="F9" t="s">
+        <v>170</v>
+      </c>
+      <c r="G9" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>189</v>
+      </c>
+      <c r="B10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" t="s">
+        <v>192</v>
+      </c>
+      <c r="D10" t="s">
+        <v>110</v>
+      </c>
+      <c r="E10" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10" t="s">
+        <v>44</v>
+      </c>
+      <c r="G10" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>189</v>
+      </c>
+      <c r="B11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" t="s">
+        <v>192</v>
+      </c>
+      <c r="D11" t="s">
+        <v>112</v>
+      </c>
+      <c r="E11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F11" t="s">
+        <v>45</v>
+      </c>
+      <c r="G11" t="s">
+        <v>173</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="32" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" t="s">
+        <v>194</v>
+      </c>
+      <c r="D2" t="s">
+        <v>106</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>108</v>
+      </c>
+      <c r="G2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>193</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>194</v>
+      </c>
+      <c r="D3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>193</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>194</v>
+      </c>
+      <c r="D4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>193</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>194</v>
+      </c>
+      <c r="D5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" t="s">
+        <v>41</v>
+      </c>
+      <c r="F5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G5" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>193</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>194</v>
+      </c>
+      <c r="D6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" t="s">
+        <v>107</v>
+      </c>
+      <c r="F6" t="s">
+        <v>36</v>
+      </c>
+      <c r="G6" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>193</v>
+      </c>
+      <c r="B7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" t="s">
+        <v>194</v>
+      </c>
+      <c r="D7" t="s">
+        <v>43</v>
+      </c>
+      <c r="E7" t="s">
+        <v>45</v>
+      </c>
+      <c r="F7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G7" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>193</v>
+      </c>
+      <c r="B8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" t="s">
+        <v>195</v>
+      </c>
+      <c r="D8" t="s">
+        <v>110</v>
+      </c>
+      <c r="E8" t="s">
+        <v>28</v>
+      </c>
+      <c r="F8" t="s">
+        <v>50</v>
+      </c>
+      <c r="G8" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>193</v>
+      </c>
+      <c r="B9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" t="s">
+        <v>195</v>
+      </c>
+      <c r="D9" t="s">
+        <v>110</v>
+      </c>
+      <c r="E9" t="s">
+        <v>172</v>
+      </c>
+      <c r="F9" t="s">
+        <v>23</v>
+      </c>
+      <c r="G9" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>193</v>
+      </c>
+      <c r="B10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" t="s">
+        <v>195</v>
+      </c>
+      <c r="D10" t="s">
+        <v>112</v>
+      </c>
+      <c r="E10" t="s">
+        <v>44</v>
+      </c>
+      <c r="F10" t="s">
+        <v>31</v>
+      </c>
+      <c r="G10" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>193</v>
+      </c>
+      <c r="B11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" t="s">
+        <v>196</v>
+      </c>
+      <c r="D11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E11" t="s">
+        <v>170</v>
+      </c>
+      <c r="F11" t="s">
+        <v>19</v>
+      </c>
+      <c r="G11" t="s">
+        <v>173</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="32" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>197</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" t="s">
+        <v>198</v>
+      </c>
+      <c r="D2" t="s">
+        <v>106</v>
+      </c>
+      <c r="E2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>197</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>198</v>
+      </c>
+      <c r="D3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" t="s">
+        <v>44</v>
+      </c>
+      <c r="G3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>197</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>198</v>
+      </c>
+      <c r="D4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E4" t="s">
+        <v>40</v>
+      </c>
+      <c r="F4" t="s">
+        <v>172</v>
+      </c>
+      <c r="G4" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>197</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>198</v>
+      </c>
+      <c r="D5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G5" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>197</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>198</v>
+      </c>
+      <c r="D6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" t="s">
+        <v>25</v>
+      </c>
+      <c r="G6" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>197</v>
+      </c>
+      <c r="B7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" t="s">
+        <v>199</v>
+      </c>
+      <c r="D7" t="s">
+        <v>110</v>
+      </c>
+      <c r="E7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" t="s">
+        <v>107</v>
+      </c>
+      <c r="G7" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>197</v>
+      </c>
+      <c r="B8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" t="s">
+        <v>199</v>
+      </c>
+      <c r="D8" t="s">
+        <v>110</v>
+      </c>
+      <c r="E8" t="s">
+        <v>36</v>
+      </c>
+      <c r="F8" t="s">
+        <v>28</v>
+      </c>
+      <c r="G8" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>197</v>
+      </c>
+      <c r="B9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" t="s">
+        <v>199</v>
+      </c>
+      <c r="D9" t="s">
+        <v>110</v>
+      </c>
+      <c r="E9" t="s">
+        <v>108</v>
+      </c>
+      <c r="F9" t="s">
+        <v>45</v>
+      </c>
+      <c r="G9" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>197</v>
+      </c>
+      <c r="B10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" t="s">
+        <v>199</v>
+      </c>
+      <c r="D10" t="s">
+        <v>112</v>
+      </c>
+      <c r="E10" t="s">
+        <v>50</v>
+      </c>
+      <c r="F10" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>197</v>
+      </c>
+      <c r="B11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" t="s">
+        <v>200</v>
+      </c>
+      <c r="D11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E11" t="s">
+        <v>18</v>
+      </c>
+      <c r="F11" t="s">
+        <v>170</v>
+      </c>
+      <c r="G11" t="s">
+        <v>173</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="32" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>201</v>
+      </c>
+      <c r="B2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C2" t="s">
+        <v>202</v>
+      </c>
+      <c r="D2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>201</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>203</v>
+      </c>
+      <c r="D3" t="s">
+        <v>106</v>
+      </c>
+      <c r="E3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>201</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>203</v>
+      </c>
+      <c r="D4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>201</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>203</v>
+      </c>
+      <c r="D5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" t="s">
+        <v>170</v>
+      </c>
+      <c r="F5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G5" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>201</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>203</v>
+      </c>
+      <c r="D6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" t="s">
+        <v>44</v>
+      </c>
+      <c r="F6" t="s">
+        <v>36</v>
+      </c>
+      <c r="G6" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>201</v>
+      </c>
+      <c r="B7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" t="s">
+        <v>203</v>
+      </c>
+      <c r="D7" t="s">
+        <v>43</v>
+      </c>
+      <c r="E7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G7" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>201</v>
+      </c>
+      <c r="B8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" t="s">
+        <v>204</v>
+      </c>
+      <c r="D8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E8" t="s">
+        <v>28</v>
+      </c>
+      <c r="F8" t="s">
+        <v>19</v>
+      </c>
+      <c r="G8" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>201</v>
+      </c>
+      <c r="B9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" t="s">
+        <v>204</v>
+      </c>
+      <c r="D9" t="s">
+        <v>39</v>
+      </c>
+      <c r="E9" t="s">
+        <v>172</v>
+      </c>
+      <c r="F9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G9" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>201</v>
+      </c>
+      <c r="B10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" t="s">
+        <v>204</v>
+      </c>
+      <c r="D10" t="s">
+        <v>39</v>
+      </c>
+      <c r="E10" t="s">
+        <v>45</v>
+      </c>
+      <c r="F10" t="s">
+        <v>22</v>
+      </c>
+      <c r="G10" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>201</v>
+      </c>
+      <c r="B11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" t="s">
+        <v>204</v>
+      </c>
+      <c r="D11" t="s">
+        <v>43</v>
+      </c>
+      <c r="E11" t="s">
+        <v>107</v>
+      </c>
+      <c r="F11" t="s">
+        <v>108</v>
+      </c>
+      <c r="G11" t="s">
+        <v>173</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="32" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>205</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" t="s">
+        <v>206</v>
+      </c>
+      <c r="D2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2" t="s">
+        <v>45</v>
+      </c>
+      <c r="G2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>205</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>206</v>
+      </c>
+      <c r="D3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" t="s">
+        <v>108</v>
+      </c>
+      <c r="G3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>205</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>206</v>
+      </c>
+      <c r="D4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" t="s">
+        <v>50</v>
+      </c>
+      <c r="G4" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>205</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>206</v>
+      </c>
+      <c r="D5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" t="s">
+        <v>170</v>
+      </c>
+      <c r="F5" t="s">
+        <v>107</v>
+      </c>
+      <c r="G5" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>205</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>206</v>
+      </c>
+      <c r="D6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" t="s">
+        <v>172</v>
+      </c>
+      <c r="F6" t="s">
+        <v>41</v>
+      </c>
+      <c r="G6" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>205</v>
+      </c>
+      <c r="B7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" t="s">
+        <v>206</v>
+      </c>
+      <c r="D7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>205</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" t="s">
+        <v>206</v>
+      </c>
+      <c r="D8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" t="s">
+        <v>28</v>
+      </c>
+      <c r="G8" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>205</v>
+      </c>
+      <c r="B9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" t="s">
+        <v>207</v>
+      </c>
+      <c r="D9" t="s">
+        <v>39</v>
+      </c>
+      <c r="E9" t="s">
+        <v>25</v>
+      </c>
+      <c r="F9" t="s">
+        <v>40</v>
+      </c>
+      <c r="G9" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>205</v>
+      </c>
+      <c r="B10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" t="s">
+        <v>207</v>
+      </c>
+      <c r="D10" t="s">
+        <v>43</v>
+      </c>
+      <c r="E10" t="s">
+        <v>44</v>
+      </c>
+      <c r="F10" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>205</v>
+      </c>
+      <c r="B11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" t="s">
+        <v>208</v>
+      </c>
+      <c r="D11" t="s">
+        <v>48</v>
+      </c>
+      <c r="E11" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" t="s">
+        <v>23</v>
+      </c>
+      <c r="G11" t="s">
+        <v>173</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="32" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" t="s">
+        <v>210</v>
+      </c>
+      <c r="D2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>172</v>
+      </c>
+      <c r="G2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>209</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>210</v>
+      </c>
+      <c r="D3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>209</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>210</v>
+      </c>
+      <c r="D4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" t="s">
+        <v>44</v>
+      </c>
+      <c r="G4" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>209</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>210</v>
+      </c>
+      <c r="D5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5" t="s">
+        <v>170</v>
+      </c>
+      <c r="G5" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>209</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>210</v>
+      </c>
+      <c r="D6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G6" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>209</v>
+      </c>
+      <c r="B7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" t="s">
+        <v>210</v>
+      </c>
+      <c r="D7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" t="s">
+        <v>41</v>
+      </c>
+      <c r="F7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G7" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>209</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" t="s">
+        <v>210</v>
+      </c>
+      <c r="D8" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" t="s">
+        <v>108</v>
+      </c>
+      <c r="F8" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>209</v>
+      </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" t="s">
+        <v>210</v>
+      </c>
+      <c r="D9" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" t="s">
+        <v>45</v>
+      </c>
+      <c r="F9" t="s">
+        <v>25</v>
+      </c>
+      <c r="G9" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>209</v>
+      </c>
+      <c r="B10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" t="s">
+        <v>210</v>
+      </c>
+      <c r="D10" t="s">
+        <v>21</v>
+      </c>
+      <c r="E10" t="s">
+        <v>50</v>
+      </c>
+      <c r="F10" t="s">
+        <v>31</v>
+      </c>
+      <c r="G10" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>209</v>
+      </c>
+      <c r="B11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" t="s">
+        <v>210</v>
+      </c>
+      <c r="D11" t="s">
+        <v>21</v>
+      </c>
+      <c r="E11" t="s">
+        <v>107</v>
+      </c>
+      <c r="F11" t="s">
+        <v>29</v>
+      </c>
+      <c r="G11" t="s">
+        <v>173</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 

</xml_diff>